<commit_message>
feat: source-traced ROI inputs + sensitivity table
</commit_message>
<xml_diff>
--- a/excel/RetailIQ_ROI_Calculator.xlsx
+++ b/excel/RetailIQ_ROI_Calculator.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RetailIQ\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E24A62CD-9827-4F25-AAA5-BA3D23A0E004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4304BC17-E097-48C4-9CD9-4AD5D34D3EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Inputs" sheetId="1" r:id="rId1"/>
+    <sheet name="Calculations" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,15 +35,183 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+  <si>
+    <t>Total active customers</t>
+  </si>
+  <si>
+    <t>Current voucher adoption %</t>
+  </si>
+  <si>
+    <t>Target voucher adoption % (what-if)</t>
+  </si>
+  <si>
+    <t>Avg order value (BRL)</t>
+  </si>
+  <si>
+    <t>Causal churn reduction from voucher</t>
+  </si>
+  <si>
+    <t>Cost per voucher issued (BRL)</t>
+  </si>
+  <si>
+    <t>Additional customers to target</t>
+  </si>
+  <si>
+    <t>Additional vouchers needed</t>
+  </si>
+  <si>
+    <t>Voucher program cost</t>
+  </si>
+  <si>
+    <t>Customers retained due to vouchers</t>
+  </si>
+  <si>
+    <t>Assumed repeat orders/year</t>
+  </si>
+  <si>
+    <t>Revenue retained (annualized)</t>
+  </si>
+  <si>
+    <t>Net ROI</t>
+  </si>
+  <si>
+    <t>Additional Customers Retained</t>
+  </si>
+  <si>
+    <t>Voucher Program Cost (BRL)</t>
+  </si>
+  <si>
+    <t>Revenue Retained (BRL)</t>
+  </si>
+  <si>
+    <t>Net ROI (BRL)</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Assumed repeat orders/year (retained customer)</t>
+  </si>
+  <si>
+    <t>Assumptions: cost/voucher and repeat-orders/year are estimates for</t>
+  </si>
+  <si>
+    <t>illustration; causal churn reduction is the measured DoWhy estimate</t>
+  </si>
+  <si>
+    <t>from notebooks/19_causal_model_dowhy.ipynb.</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <r>
+      <t>customer_features</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table, COUNT(customer_unique_id)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>treatment_voucher</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mean, Day 8</t>
+    </r>
+  </si>
+  <si>
+    <t>Assumption (what-if scenario)</t>
+  </si>
+  <si>
+    <r>
+      <t>payments_clean</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, AVG(payment_value)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DoWhy estimate, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>notebooks/19_causal_model_dowhy.ipynb</t>
+    </r>
+  </si>
+  <si>
+    <t>Assumption</t>
+  </si>
+  <si>
+    <t>Assumption (conservative, given low overall repeat rate — see Week 1 findings)</t>
+  </si>
+  <si>
+    <t>Repeat orders/year</t>
+  </si>
+  <si>
+    <t>(formula referencing that scenario)</t>
+  </si>
+  <si>
+    <t>637,800 (your current baseline)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -64,8 +234,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,9 +558,297 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E70B49-B854-4590-8142-254105CF08A8}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>96096</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>3.8800000000000001E-2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0.3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>154.11369999999999</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.17480000000000001</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8">
+        <v>1.5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0298DE61-AEDE-43EE-8E8B-D80190873088}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <f>Inputs!B2*(Inputs!B4-Inputs!B3)</f>
+        <v>25100.2752</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <f>B2</f>
+        <v>25100.2752</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <f>B3*Inputs!B7</f>
+        <v>376504.12800000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <f>B2*Inputs!B6</f>
+        <v>4387.5281049599998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <f>B5*Inputs!B5*Calculations!B6</f>
+        <v>1014267.2851640608</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1">
+        <f>B7-B4</f>
+        <v>637763.15716406074</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>1</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>2</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1CC8E11-81C0-4D9C-A7EF-65B0981625F5}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2">
+        <f>Calculations!B5</f>
+        <v>4387.5281049599998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1">
+        <f>Calculations!B4</f>
+        <v>376504.12800000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4">
+        <f>Calculations!B7</f>
+        <v>1014267.2851640608</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <f>Calculations!B8</f>
+        <v>637763.15716406074</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
style: formatting, sheet protection, assumptions documentation
</commit_message>
<xml_diff>
--- a/excel/RetailIQ_ROI_Calculator.xlsx
+++ b/excel/RetailIQ_ROI_Calculator.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RetailIQ\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81871FA6-E251-407D-B849-4351E8F66FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90700720-3C2C-4E5B-8BC0-254ED2606283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Calculations" sheetId="2" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
+    <sheet name="Assumptions &amp; Notes" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
   <si>
     <t>Total active customers</t>
   </si>
@@ -200,6 +201,57 @@
   </si>
   <si>
     <t>Selected Scenario</t>
+  </si>
+  <si>
+    <t>RetailIQ ROI Calculator — Assumptions &amp; Notes</t>
+  </si>
+  <si>
+    <t>1. Causal churn reduction (17.48%) is a measured result from a DoWhy causal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   model (propensity score matching), controlling for purchase frequency,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   review score, and delivery experience as confounders. See</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   notebooks/19_causal_model_dowhy.ipynb for the full analysis and refutation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   tests.</t>
+  </si>
+  <si>
+    <t>2. Cost per voucher (15 BRL) and repeat-orders/year (1.5, conservative given</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   this dataset's low baseline repeat-purchase rate) are illustrative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   assumptions, not measured values. Adjust these in the Inputs sheet to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   test different scenarios -- the Sensitivity table shows how Net ROI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   changes across a range of repeat-order assumptions.</t>
+  </si>
+  <si>
+    <t>3. This calculator assumes voucher adoption can be scaled linearly to the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   target % without diminishing returns -- in reality, the causal effect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   may not hold uniformly as adoption expands to customers who look</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   different from current voucher users. This is a known simplification.</t>
+  </si>
+  <si>
+    <t>4. All monetary figures are in BRL (Brazilian Real), matching the source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   dataset's currency.</t>
   </si>
 </sst>
 </file>
@@ -260,7 +312,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -581,7 +633,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="66.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -953,4 +1005,102 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0FE657F-859C-489D-BF73-F9543F615885}">
+  <dimension ref="A1:A21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="66.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test: Excel vs Python causal model reconciliation
</commit_message>
<xml_diff>
--- a/excel/RetailIQ_ROI_Calculator.xlsx
+++ b/excel/RetailIQ_ROI_Calculator.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RetailIQ\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AD8F6C4-0280-4DB1-99B5-D985B3C462A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9A59B9-CB4C-4C8F-B388-ECEC5B8AF84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Calculations" sheetId="2" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
-    <sheet name="Assumptions &amp; Notes" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId4"/>
+    <sheet name="Assumptions &amp; Notes" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="86">
   <si>
     <t>Total active customers</t>
   </si>
@@ -252,6 +253,96 @@
   </si>
   <si>
     <t xml:space="preserve">   dataset's currency.</t>
+  </si>
+  <si>
+    <t>RECONCILIATION CHECK -- run these against Power BI visuals</t>
+  </si>
+  <si>
+    <t>============================================================</t>
+  </si>
+  <si>
+    <t>Total customers (customer_features): 93397</t>
+  </si>
+  <si>
+    <t>Total revenue (all payments): 16008872.12</t>
+  </si>
+  <si>
+    <t>Overall churn rate: 80.16%</t>
+  </si>
+  <si>
+    <t>Segment counts:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                segment      n</t>
+  </si>
+  <si>
+    <t>0        Lost / Churned  23843</t>
+  </si>
+  <si>
+    <t>1             Champions  23672</t>
+  </si>
+  <si>
+    <t>2  At Risk (High Value)  22836</t>
+  </si>
+  <si>
+    <t>3       Needs Attention  11605</t>
+  </si>
+  <si>
+    <t>4       Loyal Customers  11401</t>
+  </si>
+  <si>
+    <t>Cohort month_index=0 all at 100%: True</t>
+  </si>
+  <si>
+    <t>Top 5 sellers by revenue:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                          seller_id  total_sales</t>
+  </si>
+  <si>
+    <t>0  4869f7a5dfa277a7dca6462dcf3b52b2    229472.63</t>
+  </si>
+  <si>
+    <t>1  53243585a1d6dc2643021fd1853d8905    222776.05</t>
+  </si>
+  <si>
+    <t>2  4a3ca9315b744ce9f8e9374361493884    200472.92</t>
+  </si>
+  <si>
+    <t>3  fa1c13f2614d7b5c4749cbc52fecda94    194042.03</t>
+  </si>
+  <si>
+    <t>4  7c67e1448b00f6e969d365cea6b010ab    187923.89</t>
+  </si>
+  <si>
+    <t>Top 5 states by revenue:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  customer_state  total_revenue</t>
+  </si>
+  <si>
+    <t>0             SP     5770266.19</t>
+  </si>
+  <si>
+    <t>1             RJ     2055690.45</t>
+  </si>
+  <si>
+    <t>2             MG     1819277.61</t>
+  </si>
+  <si>
+    <t>3             RS      861802.40</t>
+  </si>
+  <si>
+    <t>4             PR      781919.55</t>
+  </si>
+  <si>
+    <t>Last reconciled against notebooks/19_causal_model_dowhy.ipynb and</t>
+  </si>
+  <si>
+    <t>to match source notebooks.</t>
+  </si>
+  <si>
+    <t>docs/model_metrics.json on 03/08/2026. All input values manually verified</t>
   </si>
 </sst>
 </file>
@@ -1008,8 +1099,156 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E8C2BF-090A-429F-A960-96619A5D12AB}">
+  <dimension ref="A1:A32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="62.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0FE657F-859C-489D-BF73-F9543F615885}">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="69.6640625" customWidth="1"/>
@@ -1100,6 +1339,21 @@
         <v>55</v>
       </c>
     </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: rebuild ROI model and add proactive targeting framework
</commit_message>
<xml_diff>
--- a/excel/RetailIQ_ROI_Calculator.xlsx
+++ b/excel/RetailIQ_ROI_Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RetailIQ\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9A59B9-CB4C-4C8F-B388-ECEC5B8AF84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B0D313-9BAC-4F5A-B5D4-DA9F951BBB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{8826B70C-D4BC-40BC-92ED-3870D25B85D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="93">
   <si>
     <t>Total active customers</t>
   </si>
@@ -344,12 +344,36 @@
   <si>
     <t>docs/model_metrics.json on 03/08/2026. All input values manually verified</t>
   </si>
+  <si>
+    <t>High-risk, untreated customers (top 20% churn risk)</t>
+  </si>
+  <si>
+    <t>Avg CLV of high-risk group (BRL)</t>
+  </si>
+  <si>
+    <t>Avg predicted churn probability (high-risk group)</t>
+  </si>
+  <si>
+    <t>Cost per proactive intervention (BRL)</t>
+  </si>
+  <si>
+    <t>Addressable revenue at risk</t>
+  </si>
+  <si>
+    <t>Proactive program cost</t>
+  </si>
+  <si>
+    <t>Break-even success rate</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,6 +395,13 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -389,10 +420,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -406,9 +438,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -816,6 +850,38 @@
         <v>30</v>
       </c>
     </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9">
+        <v>18021</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10">
+        <v>183.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11">
+        <v>0.7984</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
+    </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
@@ -838,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0298DE61-AEDE-43EE-8E8B-D80190873088}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.88671875" bestFit="1" customWidth="1"/>
@@ -995,6 +1061,33 @@
       </c>
       <c r="B14" s="4">
         <v>415447.05377765995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16">
+        <f>Inputs!B9*Inputs!B10*Inputs!B11</f>
+        <v>2643788.8259999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="1">
+        <f>Inputs!B9*Inputs!B12</f>
+        <v>270315</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="7">
+        <f>B17/B16</f>
+        <v>0.10224530694041144</v>
       </c>
     </row>
   </sheetData>
@@ -1013,8 +1106,8 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1081,8 +1174,8 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="str">
-        <f>CONCATENATE("At ", TEXT(Inputs!B4,"0%")," voucher adoption (", Calculations!E2, " scenario), projected net ROI is ", TEXT(Calculations!B8,"#,##0")," BRL, retaining ", TEXT(Calculations!B5,"#,##0")," customers.")</f>
-        <v>At 15% voucher adoption (Conservative scenario), projected net ROI is 2,71,513 BRL, retaining 1,868 customers.</v>
+        <f>"Targeting the "&amp;TEXT(Inputs!B9,"#,##0")&amp;" highest-risk, currently-untargeted customers exposes "&amp;TEXT(Calculations!B16,"#,##0")&amp;" BRL in revenue at risk, at a program cost of "&amp;TEXT(Calculations!B17,"#,##0")&amp;" BRL. The program breaks even at a "&amp;TEXT(Calculations!B18,"0.0%")&amp;" churn-prevention rate — recommend validating via A/B test before scaling."</f>
+        <v>Targeting the 18,021 highest-risk, currently-untargeted customers exposes 26,43,789 BRL in revenue at risk, at a program cost of 2,70,315 BRL. The program breaks even at a 10.2% churn-prevention rate — recommend validating via A/B test before scaling.</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>

</xml_diff>